<commit_message>
added LGM50LT sample battery cell, output organization
</commit_message>
<xml_diff>
--- a/sample_data/LGM50LT.xlsx
+++ b/sample_data/LGM50LT.xlsx
@@ -8,42 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomasdolezal/Documents/Baterky/Projects/TestProfiles/BatteryTestProfileGeneration/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEE5DB7-0445-0645-8F2D-4D3FC59F4A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D3BF92-AEFC-964B-8E4D-4275B6F0A9D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="1" r:id="rId1"/>
     <sheet name="OCV" sheetId="2" r:id="rId2"/>
     <sheet name="R0" sheetId="3" r:id="rId3"/>
+    <sheet name="R0_raw" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>Var1</t>
   </si>
   <si>
     <t>Var2</t>
-  </si>
-  <si>
-    <t>SOC</t>
   </si>
   <si>
     <t>voltage_V</t>
@@ -52,10 +37,13 @@
     <t>capacity_Ah</t>
   </si>
   <si>
-    <t>type</t>
+    <t>H_mm</t>
   </si>
   <si>
-    <t>H_mm</t>
+    <t>T_mm</t>
+  </si>
+  <si>
+    <t>W_mm</t>
   </si>
   <si>
     <t>weight_g</t>
@@ -64,10 +52,10 @@
     <t>nominal_energy_Wh</t>
   </si>
   <si>
-    <t>W_mm</t>
+    <t>type</t>
   </si>
   <si>
-    <t>T_mm</t>
+    <t>cylindrical</t>
   </si>
   <si>
     <t>max_current_charge_A</t>
@@ -76,13 +64,13 @@
     <t>max_current_discharge_A</t>
   </si>
   <si>
+    <t>SOC</t>
+  </si>
+  <si>
     <t>OCV_V</t>
   </si>
   <si>
     <t>R0</t>
-  </si>
-  <si>
-    <t>cylindrical</t>
   </si>
 </sst>
 </file>
@@ -182,14 +170,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -513,132 +500,87 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>3</v>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>2</v>
       </c>
       <c r="B2" s="2">
         <v>3.69</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
-        <v>4</v>
+      <c r="A3" s="8" t="s">
+        <v>3</v>
       </c>
       <c r="B3" s="2">
         <v>4.8</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>6</v>
+    </row>
+    <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="B4" s="2">
         <v>70.650000000000006</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>10</v>
+    </row>
+    <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>5</v>
       </c>
       <c r="B5" s="2">
         <v>21.44</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>9</v>
+    </row>
+    <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>6</v>
       </c>
       <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2">
         <v>67.5</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="2">
         <v>18.2</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
-        <v>5</v>
+      <c r="A9" s="8" t="s">
+        <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+        <v>10</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="5">
-        <v>2.36</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
+      <c r="B10" s="4">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>14.4</v>
       </c>
     </row>
@@ -653,1619 +595,1619 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>13</v>
       </c>
+      <c r="B1" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="6">
+      <c r="A2" s="5">
         <v>0</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="5">
         <v>2.58765</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="6">
+      <c r="A3" s="5">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="5">
         <v>2.7979883000000001</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>0.01</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2.9229349999999998</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="6">
+      <c r="A5" s="5">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <v>3.0058137999999999</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="6">
+      <c r="A6" s="5">
         <v>0.02</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <v>3.0700850000000002</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="6">
+      <c r="A7" s="5">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <v>3.1224763000000002</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="6">
+      <c r="A8" s="5">
         <v>0.03</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <v>3.166849</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="6">
+      <c r="A9" s="5">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="5">
         <v>3.2053284999999998</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="6">
+      <c r="A10" s="5">
         <v>0.04</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="5">
         <v>3.239204</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="6">
+      <c r="A11" s="5">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="5">
         <v>3.2694117999999999</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="6">
+      <c r="A12" s="5">
         <v>0.05</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="5">
         <v>3.2965100000000001</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="6">
+      <c r="A13" s="5">
         <v>5.5E-2</v>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="5">
         <v>3.3208760000000002</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="6">
+      <c r="A14" s="5">
         <v>0.06</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="5">
         <v>3.3421569999999998</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="6">
+      <c r="A15" s="5">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="5">
         <v>3.3587867999999999</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="6">
+      <c r="A16" s="5">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="5">
         <v>3.3693165</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="6">
+      <c r="A17" s="5">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="5">
         <v>3.3761000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="6">
+      <c r="A18" s="5">
         <v>0.08</v>
       </c>
-      <c r="B18" s="6">
+      <c r="B18" s="5">
         <v>3.3816000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="6">
+      <c r="A19" s="5">
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="5">
         <v>3.3865219999999998</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="6">
+      <c r="A20" s="5">
         <v>0.09</v>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="5">
         <v>3.3911644999999999</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="6">
+      <c r="A21" s="5">
         <v>9.5000000000000001E-2</v>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="5">
         <v>3.39575</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="6">
+      <c r="A22" s="5">
         <v>0.1</v>
       </c>
-      <c r="B22" s="6">
+      <c r="B22" s="5">
         <v>3.40015</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="6">
+      <c r="A23" s="5">
         <v>0.105</v>
       </c>
-      <c r="B23" s="6">
+      <c r="B23" s="5">
         <v>3.4045747999999998</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="6">
+      <c r="A24" s="5">
         <v>0.11</v>
       </c>
-      <c r="B24" s="6">
+      <c r="B24" s="5">
         <v>3.4089999999999998</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="6">
+      <c r="A25" s="5">
         <v>0.115</v>
       </c>
-      <c r="B25" s="6">
+      <c r="B25" s="5">
         <v>3.4135</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="6">
+      <c r="A26" s="5">
         <v>0.12</v>
       </c>
-      <c r="B26" s="6">
+      <c r="B26" s="5">
         <v>3.41805</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="6">
+      <c r="A27" s="5">
         <v>0.125</v>
       </c>
-      <c r="B27" s="6">
+      <c r="B27" s="5">
         <v>3.4228562999999999</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="6">
+      <c r="A28" s="5">
         <v>0.13</v>
       </c>
-      <c r="B28" s="6">
+      <c r="B28" s="5">
         <v>3.4279999999999999</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="6">
+      <c r="A29" s="5">
         <v>0.13500000000000001</v>
       </c>
-      <c r="B29" s="6">
+      <c r="B29" s="5">
         <v>3.4336820000000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" s="6">
+      <c r="A30" s="5">
         <v>0.14000000000000001</v>
       </c>
-      <c r="B30" s="6">
+      <c r="B30" s="5">
         <v>3.4399479999999998</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="6">
+      <c r="A31" s="5">
         <v>0.14499999999999999</v>
       </c>
-      <c r="B31" s="6">
+      <c r="B31" s="5">
         <v>3.4465140000000001</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="6">
+      <c r="A32" s="5">
         <v>0.15</v>
       </c>
-      <c r="B32" s="6">
+      <c r="B32" s="5">
         <v>3.4532725000000002</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="6">
+      <c r="A33" s="5">
         <v>0.155</v>
       </c>
-      <c r="B33" s="6">
+      <c r="B33" s="5">
         <v>3.4598460000000002</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" s="6">
+      <c r="A34" s="5">
         <v>0.16</v>
       </c>
-      <c r="B34" s="6">
+      <c r="B34" s="5">
         <v>3.4662999999999999</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" s="6">
+      <c r="A35" s="5">
         <v>0.16500000000000001</v>
       </c>
-      <c r="B35" s="6">
+      <c r="B35" s="5">
         <v>3.4725598</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="6">
+      <c r="A36" s="5">
         <v>0.17</v>
       </c>
-      <c r="B36" s="6">
+      <c r="B36" s="5">
         <v>3.4788999999999999</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="6">
+      <c r="A37" s="5">
         <v>0.17499999999999999</v>
       </c>
-      <c r="B37" s="6">
+      <c r="B37" s="5">
         <v>3.4852500000000002</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="6">
+      <c r="A38" s="5">
         <v>0.18</v>
       </c>
-      <c r="B38" s="6">
+      <c r="B38" s="5">
         <v>3.4914999999999998</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="6">
+      <c r="A39" s="5">
         <v>0.185</v>
       </c>
-      <c r="B39" s="6">
+      <c r="B39" s="5">
         <v>3.4976500000000001</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" s="6">
+      <c r="A40" s="5">
         <v>0.19</v>
       </c>
-      <c r="B40" s="6">
+      <c r="B40" s="5">
         <v>3.5032580000000002</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" s="6">
+      <c r="A41" s="5">
         <v>0.19500000000000001</v>
       </c>
-      <c r="B41" s="6">
+      <c r="B41" s="5">
         <v>3.5085999999999999</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="6">
+      <c r="A42" s="5">
         <v>0.2</v>
       </c>
-      <c r="B42" s="6">
+      <c r="B42" s="5">
         <v>3.5137</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="6">
+      <c r="A43" s="5">
         <v>0.20499999999999999</v>
       </c>
-      <c r="B43" s="6">
+      <c r="B43" s="5">
         <v>3.5186500000000001</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" s="6">
+      <c r="A44" s="5">
         <v>0.21</v>
       </c>
-      <c r="B44" s="6">
+      <c r="B44" s="5">
         <v>3.5235715000000001</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" s="6">
+      <c r="A45" s="5">
         <v>0.215</v>
       </c>
-      <c r="B45" s="6">
+      <c r="B45" s="5">
         <v>3.5286499999999998</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" s="6">
+      <c r="A46" s="5">
         <v>0.22</v>
       </c>
-      <c r="B46" s="6">
+      <c r="B46" s="5">
         <v>3.533709</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" s="6">
+      <c r="A47" s="5">
         <v>0.22500000000000001</v>
       </c>
-      <c r="B47" s="6">
+      <c r="B47" s="5">
         <v>3.5388000000000002</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" s="6">
+      <c r="A48" s="5">
         <v>0.23</v>
       </c>
-      <c r="B48" s="6">
+      <c r="B48" s="5">
         <v>3.5437500000000002</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" s="6">
+      <c r="A49" s="5">
         <v>0.23499999999999999</v>
       </c>
-      <c r="B49" s="6">
+      <c r="B49" s="5">
         <v>3.5483500000000001</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" s="6">
+      <c r="A50" s="5">
         <v>0.24</v>
       </c>
-      <c r="B50" s="6">
+      <c r="B50" s="5">
         <v>3.5528</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" s="6">
+      <c r="A51" s="5">
         <v>0.245</v>
       </c>
-      <c r="B51" s="6">
+      <c r="B51" s="5">
         <v>3.5569918</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" s="6">
+      <c r="A52" s="5">
         <v>0.25</v>
       </c>
-      <c r="B52" s="6">
+      <c r="B52" s="5">
         <v>3.5611875</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" s="6">
+      <c r="A53" s="5">
         <v>0.255</v>
       </c>
-      <c r="B53" s="6">
+      <c r="B53" s="5">
         <v>3.5651660000000001</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="6">
+      <c r="A54" s="5">
         <v>0.26</v>
       </c>
-      <c r="B54" s="6">
+      <c r="B54" s="5">
         <v>3.569</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="6">
+      <c r="A55" s="5">
         <v>0.26500000000000001</v>
       </c>
-      <c r="B55" s="6">
+      <c r="B55" s="5">
         <v>3.572848</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" s="6">
+      <c r="A56" s="5">
         <v>0.27</v>
       </c>
-      <c r="B56" s="6">
+      <c r="B56" s="5">
         <v>3.5764434999999999</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57" s="6">
+      <c r="A57" s="5">
         <v>0.27500000000000002</v>
       </c>
-      <c r="B57" s="6">
+      <c r="B57" s="5">
         <v>3.5798999999999999</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A58" s="6">
+      <c r="A58" s="5">
         <v>0.28000000000000003</v>
       </c>
-      <c r="B58" s="6">
+      <c r="B58" s="5">
         <v>3.5833460000000001</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A59" s="6">
+      <c r="A59" s="5">
         <v>0.28499999999999998</v>
       </c>
-      <c r="B59" s="6">
+      <c r="B59" s="5">
         <v>3.5866457999999999</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A60" s="6">
+      <c r="A60" s="5">
         <v>0.28999999999999998</v>
       </c>
-      <c r="B60" s="6">
+      <c r="B60" s="5">
         <v>3.5898755000000002</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A61" s="6">
+      <c r="A61" s="5">
         <v>0.29499999999999998</v>
       </c>
-      <c r="B61" s="6">
+      <c r="B61" s="5">
         <v>3.5931000000000002</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A62" s="6">
+      <c r="A62" s="5">
         <v>0.3</v>
       </c>
-      <c r="B62" s="6">
+      <c r="B62" s="5">
         <v>3.5962000000000001</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A63" s="6">
+      <c r="A63" s="5">
         <v>0.30499999999999999</v>
       </c>
-      <c r="B63" s="6">
+      <c r="B63" s="5">
         <v>3.5994000000000002</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A64" s="6">
+      <c r="A64" s="5">
         <v>0.31</v>
       </c>
-      <c r="B64" s="6">
+      <c r="B64" s="5">
         <v>3.6024444999999998</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A65" s="6">
+      <c r="A65" s="5">
         <v>0.315</v>
       </c>
-      <c r="B65" s="6">
+      <c r="B65" s="5">
         <v>3.6055419999999998</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A66" s="6">
+      <c r="A66" s="5">
         <v>0.32</v>
       </c>
-      <c r="B66" s="6">
+      <c r="B66" s="5">
         <v>3.6086</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A67" s="6">
+      <c r="A67" s="5">
         <v>0.32500000000000001</v>
       </c>
-      <c r="B67" s="6">
+      <c r="B67" s="5">
         <v>3.6114999999999999</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A68" s="6">
+      <c r="A68" s="5">
         <v>0.33</v>
       </c>
-      <c r="B68" s="6">
+      <c r="B68" s="5">
         <v>3.6144634999999998</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A69" s="6">
+      <c r="A69" s="5">
         <v>0.33500000000000002</v>
       </c>
-      <c r="B69" s="6">
+      <c r="B69" s="5">
         <v>3.6173932999999998</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A70" s="6">
+      <c r="A70" s="5">
         <v>0.34</v>
       </c>
-      <c r="B70" s="6">
+      <c r="B70" s="5">
         <v>3.6202999999999999</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A71" s="6">
+      <c r="A71" s="5">
         <v>0.34499999999999997</v>
       </c>
-      <c r="B71" s="6">
+      <c r="B71" s="5">
         <v>3.6232000000000002</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A72" s="6">
+      <c r="A72" s="5">
         <v>0.35</v>
       </c>
-      <c r="B72" s="6">
+      <c r="B72" s="5">
         <v>3.6260500000000002</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A73" s="6">
+      <c r="A73" s="5">
         <v>0.35499999999999998</v>
       </c>
-      <c r="B73" s="6">
+      <c r="B73" s="5">
         <v>3.6289482999999998</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A74" s="6">
+      <c r="A74" s="5">
         <v>0.36</v>
       </c>
-      <c r="B74" s="6">
+      <c r="B74" s="5">
         <v>3.63185</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A75" s="6">
+      <c r="A75" s="5">
         <v>0.36499999999999999</v>
       </c>
-      <c r="B75" s="6">
+      <c r="B75" s="5">
         <v>3.6347217999999999</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A76" s="6">
+      <c r="A76" s="5">
         <v>0.37</v>
       </c>
-      <c r="B76" s="6">
+      <c r="B76" s="5">
         <v>3.6376339999999998</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A77" s="6">
+      <c r="A77" s="5">
         <v>0.375</v>
       </c>
-      <c r="B77" s="6">
+      <c r="B77" s="5">
         <v>3.6405500000000002</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A78" s="6">
+      <c r="A78" s="5">
         <v>0.38</v>
       </c>
-      <c r="B78" s="6">
+      <c r="B78" s="5">
         <v>3.6435050000000002</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A79" s="6">
+      <c r="A79" s="5">
         <v>0.38500000000000001</v>
       </c>
-      <c r="B79" s="6">
+      <c r="B79" s="5">
         <v>3.6464500000000002</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A80" s="6">
+      <c r="A80" s="5">
         <v>0.39</v>
       </c>
-      <c r="B80" s="6">
+      <c r="B80" s="5">
         <v>3.6494295000000001</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A81" s="6">
+      <c r="A81" s="5">
         <v>0.39500000000000002</v>
       </c>
-      <c r="B81" s="6">
+      <c r="B81" s="5">
         <v>3.6524640000000002</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A82" s="6">
+      <c r="A82" s="5">
         <v>0.4</v>
       </c>
-      <c r="B82" s="6">
+      <c r="B82" s="5">
         <v>3.6555200000000001</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A83" s="6">
+      <c r="A83" s="5">
         <v>0.40500000000000003</v>
       </c>
-      <c r="B83" s="6">
+      <c r="B83" s="5">
         <v>3.6586539999999999</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A84" s="6">
+      <c r="A84" s="5">
         <v>0.41</v>
       </c>
-      <c r="B84" s="6">
+      <c r="B84" s="5">
         <v>3.6619000000000002</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A85" s="6">
+      <c r="A85" s="5">
         <v>0.41499999999999998</v>
       </c>
-      <c r="B85" s="6">
+      <c r="B85" s="5">
         <v>3.6650912999999998</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A86" s="6">
+      <c r="A86" s="5">
         <v>0.42</v>
       </c>
-      <c r="B86" s="6">
+      <c r="B86" s="5">
         <v>3.6684999999999999</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A87" s="6">
+      <c r="A87" s="5">
         <v>0.42499999999999999</v>
       </c>
-      <c r="B87" s="6">
+      <c r="B87" s="5">
         <v>3.67184</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A88" s="6">
+      <c r="A88" s="5">
         <v>0.43</v>
       </c>
-      <c r="B88" s="6">
+      <c r="B88" s="5">
         <v>3.675376</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A89" s="6">
+      <c r="A89" s="5">
         <v>0.435</v>
       </c>
-      <c r="B89" s="6">
+      <c r="B89" s="5">
         <v>3.6789499999999999</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A90" s="6">
+      <c r="A90" s="5">
         <v>0.44</v>
       </c>
-      <c r="B90" s="6">
+      <c r="B90" s="5">
         <v>3.6826180000000002</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A91" s="6">
+      <c r="A91" s="5">
         <v>0.44500000000000001</v>
       </c>
-      <c r="B91" s="6">
+      <c r="B91" s="5">
         <v>3.686474</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A92" s="6">
+      <c r="A92" s="5">
         <v>0.45</v>
       </c>
-      <c r="B92" s="6">
+      <c r="B92" s="5">
         <v>3.6903999999999999</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A93" s="6">
+      <c r="A93" s="5">
         <v>0.45500000000000002</v>
       </c>
-      <c r="B93" s="6">
+      <c r="B93" s="5">
         <v>3.6945000000000001</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A94" s="6">
+      <c r="A94" s="5">
         <v>0.46</v>
       </c>
-      <c r="B94" s="6">
+      <c r="B94" s="5">
         <v>3.6987000000000001</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A95" s="6">
+      <c r="A95" s="5">
         <v>0.46500000000000002</v>
       </c>
-      <c r="B95" s="6">
+      <c r="B95" s="5">
         <v>3.7030832999999999</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A96" s="6">
+      <c r="A96" s="5">
         <v>0.47</v>
       </c>
-      <c r="B96" s="6">
+      <c r="B96" s="5">
         <v>3.7075040000000001</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" s="6">
+      <c r="A97" s="5">
         <v>0.47499999999999998</v>
       </c>
-      <c r="B97" s="6">
+      <c r="B97" s="5">
         <v>3.7122000000000002</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A98" s="6">
+      <c r="A98" s="5">
         <v>0.48</v>
       </c>
-      <c r="B98" s="6">
+      <c r="B98" s="5">
         <v>3.7169500000000002</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A99" s="6">
+      <c r="A99" s="5">
         <v>0.48499999999999999</v>
       </c>
-      <c r="B99" s="6">
+      <c r="B99" s="5">
         <v>3.7219338</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A100" s="6">
+      <c r="A100" s="5">
         <v>0.49</v>
       </c>
-      <c r="B100" s="6">
+      <c r="B100" s="5">
         <v>3.7269000000000001</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A101" s="6">
+      <c r="A101" s="5">
         <v>0.495</v>
       </c>
-      <c r="B101" s="6">
+      <c r="B101" s="5">
         <v>3.7320500000000001</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A102" s="6">
+      <c r="A102" s="5">
         <v>0.5</v>
       </c>
-      <c r="B102" s="6">
+      <c r="B102" s="5">
         <v>3.7374000000000001</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A103" s="6">
+      <c r="A103" s="5">
         <v>0.505</v>
       </c>
-      <c r="B103" s="6">
+      <c r="B103" s="5">
         <v>3.7427160000000002</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A104" s="6">
+      <c r="A104" s="5">
         <v>0.51</v>
       </c>
-      <c r="B104" s="6">
+      <c r="B104" s="5">
         <v>3.7482845</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A105" s="6">
+      <c r="A105" s="5">
         <v>0.51500000000000001</v>
       </c>
-      <c r="B105" s="6">
+      <c r="B105" s="5">
         <v>3.7538143000000002</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A106" s="6">
+      <c r="A106" s="5">
         <v>0.52</v>
       </c>
-      <c r="B106" s="6">
+      <c r="B106" s="5">
         <v>3.7595499999999999</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A107" s="6">
+      <c r="A107" s="5">
         <v>0.52500000000000002</v>
       </c>
-      <c r="B107" s="6">
+      <c r="B107" s="5">
         <v>3.7654000000000001</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A108" s="6">
+      <c r="A108" s="5">
         <v>0.53</v>
       </c>
-      <c r="B108" s="6">
+      <c r="B108" s="5">
         <v>3.7713494999999999</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A109" s="6">
+      <c r="A109" s="5">
         <v>0.53500000000000003</v>
       </c>
-      <c r="B109" s="6">
+      <c r="B109" s="5">
         <v>3.7774619999999999</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A110" s="6">
+      <c r="A110" s="5">
         <v>0.54</v>
       </c>
-      <c r="B110" s="6">
+      <c r="B110" s="5">
         <v>3.783887</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A111" s="6">
+      <c r="A111" s="5">
         <v>0.54500000000000004</v>
       </c>
-      <c r="B111" s="6">
+      <c r="B111" s="5">
         <v>3.7904928</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A112" s="6">
+      <c r="A112" s="5">
         <v>0.55000000000000004</v>
       </c>
-      <c r="B112" s="6">
+      <c r="B112" s="5">
         <v>3.7973599999999998</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A113" s="6">
+      <c r="A113" s="5">
         <v>0.55500000000000005</v>
       </c>
-      <c r="B113" s="6">
+      <c r="B113" s="5">
         <v>3.8046000000000002</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A114" s="6">
+      <c r="A114" s="5">
         <v>0.56000000000000005</v>
       </c>
-      <c r="B114" s="6">
+      <c r="B114" s="5">
         <v>3.8118240000000001</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A115" s="6">
+      <c r="A115" s="5">
         <v>0.56499999999999995</v>
       </c>
-      <c r="B115" s="6">
+      <c r="B115" s="5">
         <v>3.8187000000000002</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A116" s="6">
+      <c r="A116" s="5">
         <v>0.56999999999999995</v>
       </c>
-      <c r="B116" s="6">
+      <c r="B116" s="5">
         <v>3.8252000000000002</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A117" s="6">
+      <c r="A117" s="5">
         <v>0.57499999999999996</v>
       </c>
-      <c r="B117" s="6">
+      <c r="B117" s="5">
         <v>3.8313712999999998</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A118" s="6">
+      <c r="A118" s="5">
         <v>0.57999999999999996</v>
       </c>
-      <c r="B118" s="6">
+      <c r="B118" s="5">
         <v>3.8372000000000002</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A119" s="6">
+      <c r="A119" s="5">
         <v>0.58499999999999996</v>
       </c>
-      <c r="B119" s="6">
+      <c r="B119" s="5">
         <v>3.8427720000000001</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A120" s="6">
+      <c r="A120" s="5">
         <v>0.59</v>
       </c>
-      <c r="B120" s="6">
+      <c r="B120" s="5">
         <v>3.8480604999999999</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A121" s="6">
+      <c r="A121" s="5">
         <v>0.59499999999999997</v>
       </c>
-      <c r="B121" s="6">
+      <c r="B121" s="5">
         <v>3.8532540000000002</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A122" s="6">
+      <c r="A122" s="5">
         <v>0.6</v>
       </c>
-      <c r="B122" s="6">
+      <c r="B122" s="5">
         <v>3.85825</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A123" s="6">
+      <c r="A123" s="5">
         <v>0.60499999999999998</v>
       </c>
-      <c r="B123" s="6">
+      <c r="B123" s="5">
         <v>3.8629859999999998</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A124" s="6">
+      <c r="A124" s="5">
         <v>0.61</v>
       </c>
-      <c r="B124" s="6">
+      <c r="B124" s="5">
         <v>3.8676295000000001</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A125" s="6">
+      <c r="A125" s="5">
         <v>0.61499999999999999</v>
       </c>
-      <c r="B125" s="6">
+      <c r="B125" s="5">
         <v>3.8721179999999999</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A126" s="6">
+      <c r="A126" s="5">
         <v>0.62</v>
       </c>
-      <c r="B126" s="6">
+      <c r="B126" s="5">
         <v>3.8764500000000002</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A127" s="6">
+      <c r="A127" s="5">
         <v>0.625</v>
       </c>
-      <c r="B127" s="6">
+      <c r="B127" s="5">
         <v>3.8807</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A128" s="6">
+      <c r="A128" s="5">
         <v>0.63</v>
       </c>
-      <c r="B128" s="6">
+      <c r="B128" s="5">
         <v>3.8848500000000001</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A129" s="6">
+      <c r="A129" s="5">
         <v>0.63500000000000001</v>
       </c>
-      <c r="B129" s="6">
+      <c r="B129" s="5">
         <v>3.8887999999999998</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A130" s="6">
+      <c r="A130" s="5">
         <v>0.64</v>
       </c>
-      <c r="B130" s="6">
+      <c r="B130" s="5">
         <v>3.8926500000000002</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A131" s="6">
+      <c r="A131" s="5">
         <v>0.64500000000000002</v>
       </c>
-      <c r="B131" s="6">
+      <c r="B131" s="5">
         <v>3.896414</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A132" s="6">
+      <c r="A132" s="5">
         <v>0.65</v>
       </c>
-      <c r="B132" s="6">
+      <c r="B132" s="5">
         <v>3.9000499999999998</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A133" s="6">
+      <c r="A133" s="5">
         <v>0.65500000000000003</v>
       </c>
-      <c r="B133" s="6">
+      <c r="B133" s="5">
         <v>3.9036460000000002</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A134" s="6">
+      <c r="A134" s="5">
         <v>0.66</v>
       </c>
-      <c r="B134" s="6">
+      <c r="B134" s="5">
         <v>3.9071500000000001</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A135" s="6">
+      <c r="A135" s="5">
         <v>0.66500000000000004</v>
       </c>
-      <c r="B135" s="6">
+      <c r="B135" s="5">
         <v>3.9106000000000001</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A136" s="6">
+      <c r="A136" s="5">
         <v>0.67</v>
       </c>
-      <c r="B136" s="6">
+      <c r="B136" s="5">
         <v>3.914094</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A137" s="6">
+      <c r="A137" s="5">
         <v>0.67500000000000004</v>
       </c>
-      <c r="B137" s="6">
+      <c r="B137" s="5">
         <v>3.9175</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A138" s="6">
+      <c r="A138" s="5">
         <v>0.68</v>
       </c>
-      <c r="B138" s="6">
+      <c r="B138" s="5">
         <v>3.9209260000000001</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A139" s="6">
+      <c r="A139" s="5">
         <v>0.68500000000000005</v>
       </c>
-      <c r="B139" s="6">
+      <c r="B139" s="5">
         <v>3.9245000000000001</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A140" s="6">
+      <c r="A140" s="5">
         <v>0.69</v>
       </c>
-      <c r="B140" s="6">
+      <c r="B140" s="5">
         <v>3.9281000000000001</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A141" s="6">
+      <c r="A141" s="5">
         <v>0.69499999999999995</v>
       </c>
-      <c r="B141" s="6">
+      <c r="B141" s="5">
         <v>3.9318499999999998</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A142" s="6">
+      <c r="A142" s="5">
         <v>0.7</v>
       </c>
-      <c r="B142" s="6">
+      <c r="B142" s="5">
         <v>3.93574</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A143" s="6">
+      <c r="A143" s="5">
         <v>0.70499999999999996</v>
       </c>
-      <c r="B143" s="6">
+      <c r="B143" s="5">
         <v>3.9397500000000001</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A144" s="6">
+      <c r="A144" s="5">
         <v>0.71</v>
       </c>
-      <c r="B144" s="6">
+      <c r="B144" s="5">
         <v>3.9439500000000001</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A145" s="6">
+      <c r="A145" s="5">
         <v>0.71499999999999997</v>
       </c>
-      <c r="B145" s="6">
+      <c r="B145" s="5">
         <v>3.94835</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A146" s="6">
+      <c r="A146" s="5">
         <v>0.72</v>
       </c>
-      <c r="B146" s="6">
+      <c r="B146" s="5">
         <v>3.9529839999999998</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A147" s="6">
+      <c r="A147" s="5">
         <v>0.72499999999999998</v>
       </c>
-      <c r="B147" s="6">
+      <c r="B147" s="5">
         <v>3.9578000000000002</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A148" s="6">
+      <c r="A148" s="5">
         <v>0.73</v>
       </c>
-      <c r="B148" s="6">
+      <c r="B148" s="5">
         <v>3.9628359999999998</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A149" s="6">
+      <c r="A149" s="5">
         <v>0.73499999999999999</v>
       </c>
-      <c r="B149" s="6">
+      <c r="B149" s="5">
         <v>3.9681000000000002</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A150" s="6">
+      <c r="A150" s="5">
         <v>0.74</v>
       </c>
-      <c r="B150" s="6">
+      <c r="B150" s="5">
         <v>3.9735499999999999</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A151" s="6">
+      <c r="A151" s="5">
         <v>0.745</v>
       </c>
-      <c r="B151" s="6">
+      <c r="B151" s="5">
         <v>3.9790999999999999</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A152" s="6">
+      <c r="A152" s="5">
         <v>0.75</v>
       </c>
-      <c r="B152" s="6">
+      <c r="B152" s="5">
         <v>3.9849999999999999</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A153" s="6">
+      <c r="A153" s="5">
         <v>0.755</v>
       </c>
-      <c r="B153" s="6">
+      <c r="B153" s="5">
         <v>3.990866</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A154" s="6">
+      <c r="A154" s="5">
         <v>0.76</v>
       </c>
-      <c r="B154" s="6">
+      <c r="B154" s="5">
         <v>3.996972</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A155" s="6">
+      <c r="A155" s="5">
         <v>0.76500000000000001</v>
       </c>
-      <c r="B155" s="6">
+      <c r="B155" s="5">
         <v>4.0031999999999996</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A156" s="6">
+      <c r="A156" s="5">
         <v>0.77</v>
       </c>
-      <c r="B156" s="6">
+      <c r="B156" s="5">
         <v>4.0094314999999998</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A157" s="6">
+      <c r="A157" s="5">
         <v>0.77500000000000002</v>
       </c>
-      <c r="B157" s="6">
+      <c r="B157" s="5">
         <v>4.0155799999999999</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A158" s="6">
+      <c r="A158" s="5">
         <v>0.78</v>
       </c>
-      <c r="B158" s="6">
+      <c r="B158" s="5">
         <v>4.0217409999999996</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A159" s="6">
+      <c r="A159" s="5">
         <v>0.78500000000000003</v>
       </c>
-      <c r="B159" s="6">
+      <c r="B159" s="5">
         <v>4.0277327999999999</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A160" s="6">
+      <c r="A160" s="5">
         <v>0.79</v>
       </c>
-      <c r="B160" s="6">
+      <c r="B160" s="5">
         <v>4.03355</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A161" s="6">
+      <c r="A161" s="5">
         <v>0.79500000000000004</v>
       </c>
-      <c r="B161" s="6">
+      <c r="B161" s="5">
         <v>4.0391743</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A162" s="6">
+      <c r="A162" s="5">
         <v>0.8</v>
       </c>
-      <c r="B162" s="6">
+      <c r="B162" s="5">
         <v>4.0444599999999999</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A163" s="6">
+      <c r="A163" s="5">
         <v>0.80500000000000005</v>
       </c>
-      <c r="B163" s="6">
+      <c r="B163" s="5">
         <v>4.0495897999999997</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A164" s="6">
+      <c r="A164" s="5">
         <v>0.81</v>
       </c>
-      <c r="B164" s="6">
+      <c r="B164" s="5">
         <v>4.0544419999999999</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A165" s="6">
+      <c r="A165" s="5">
         <v>0.81499999999999995</v>
       </c>
-      <c r="B165" s="6">
+      <c r="B165" s="5">
         <v>4.0588499999999996</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A166" s="6">
+      <c r="A166" s="5">
         <v>0.82</v>
       </c>
-      <c r="B166" s="6">
+      <c r="B166" s="5">
         <v>4.0630499999999996</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A167" s="6">
+      <c r="A167" s="5">
         <v>0.82499999999999996</v>
       </c>
-      <c r="B167" s="6">
+      <c r="B167" s="5">
         <v>4.0667999999999997</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A168" s="6">
+      <c r="A168" s="5">
         <v>0.83</v>
       </c>
-      <c r="B168" s="6">
+      <c r="B168" s="5">
         <v>4.0701115000000003</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A169" s="6">
+      <c r="A169" s="5">
         <v>0.83499999999999996</v>
       </c>
-      <c r="B169" s="6">
+      <c r="B169" s="5">
         <v>4.0730500000000003</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A170" s="6">
+      <c r="A170" s="5">
         <v>0.84</v>
       </c>
-      <c r="B170" s="6">
+      <c r="B170" s="5">
         <v>4.07545</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A171" s="6">
+      <c r="A171" s="5">
         <v>0.84499999999999997</v>
       </c>
-      <c r="B171" s="6">
+      <c r="B171" s="5">
         <v>4.0775722999999999</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A172" s="6">
+      <c r="A172" s="5">
         <v>0.85</v>
       </c>
-      <c r="B172" s="6">
+      <c r="B172" s="5">
         <v>4.07925</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A173" s="6">
+      <c r="A173" s="5">
         <v>0.85499999999999998</v>
       </c>
-      <c r="B173" s="6">
+      <c r="B173" s="5">
         <v>4.0806627999999998</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A174" s="6">
+      <c r="A174" s="5">
         <v>0.86</v>
       </c>
-      <c r="B174" s="6">
+      <c r="B174" s="5">
         <v>4.08195</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A175" s="6">
+      <c r="A175" s="5">
         <v>0.86499999999999999</v>
       </c>
-      <c r="B175" s="6">
+      <c r="B175" s="5">
         <v>4.0830679999999999</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A176" s="6">
+      <c r="A176" s="5">
         <v>0.87</v>
       </c>
-      <c r="B176" s="6">
+      <c r="B176" s="5">
         <v>4.0841500000000002</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A177" s="6">
+      <c r="A177" s="5">
         <v>0.875</v>
       </c>
-      <c r="B177" s="6">
+      <c r="B177" s="5">
         <v>4.0852063000000003</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A178" s="6">
+      <c r="A178" s="5">
         <v>0.88</v>
       </c>
-      <c r="B178" s="6">
+      <c r="B178" s="5">
         <v>4.0861999999999998</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A179" s="6">
+      <c r="A179" s="5">
         <v>0.88500000000000001</v>
       </c>
-      <c r="B179" s="6">
+      <c r="B179" s="5">
         <v>4.0872158000000001</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A180" s="6">
+      <c r="A180" s="5">
         <v>0.89</v>
       </c>
-      <c r="B180" s="6">
+      <c r="B180" s="5">
         <v>4.0883000000000003</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A181" s="6">
+      <c r="A181" s="5">
         <v>0.89500000000000002</v>
       </c>
-      <c r="B181" s="6">
+      <c r="B181" s="5">
         <v>4.0894500000000003</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A182" s="6">
+      <c r="A182" s="5">
         <v>0.9</v>
       </c>
-      <c r="B182" s="6">
+      <c r="B182" s="5">
         <v>4.0906000000000002</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A183" s="6">
+      <c r="A183" s="5">
         <v>0.90500000000000003</v>
       </c>
-      <c r="B183" s="6">
+      <c r="B183" s="5">
         <v>4.0919153000000001</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A184" s="6">
+      <c r="A184" s="5">
         <v>0.91</v>
       </c>
-      <c r="B184" s="6">
+      <c r="B184" s="5">
         <v>4.0932620000000002</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A185" s="6">
+      <c r="A185" s="5">
         <v>0.91500000000000004</v>
       </c>
-      <c r="B185" s="6">
+      <c r="B185" s="5">
         <v>4.0947500000000003</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A186" s="6">
+      <c r="A186" s="5">
         <v>0.92</v>
       </c>
-      <c r="B186" s="6">
+      <c r="B186" s="5">
         <v>4.0964239999999998</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A187" s="6">
+      <c r="A187" s="5">
         <v>0.92500000000000004</v>
       </c>
-      <c r="B187" s="6">
+      <c r="B187" s="5">
         <v>4.0982000000000003</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A188" s="6">
+      <c r="A188" s="5">
         <v>0.93</v>
       </c>
-      <c r="B188" s="6">
+      <c r="B188" s="5">
         <v>4.10025</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A189" s="6">
+      <c r="A189" s="5">
         <v>0.93500000000000005</v>
       </c>
-      <c r="B189" s="6">
+      <c r="B189" s="5">
         <v>4.1024552999999999</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A190" s="6">
+      <c r="A190" s="5">
         <v>0.94</v>
       </c>
-      <c r="B190" s="6">
+      <c r="B190" s="5">
         <v>4.1049499999999997</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A191" s="6">
+      <c r="A191" s="5">
         <v>0.94499999999999995</v>
       </c>
-      <c r="B191" s="6">
+      <c r="B191" s="5">
         <v>4.1078000000000001</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A192" s="6">
+      <c r="A192" s="5">
         <v>0.95</v>
       </c>
-      <c r="B192" s="6">
+      <c r="B192" s="5">
         <v>4.1109</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A193" s="6">
+      <c r="A193" s="5">
         <v>0.95499999999999996</v>
       </c>
-      <c r="B193" s="6">
+      <c r="B193" s="5">
         <v>4.1144499999999997</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A194" s="6">
+      <c r="A194" s="5">
         <v>0.96</v>
       </c>
-      <c r="B194" s="6">
+      <c r="B194" s="5">
         <v>4.1184500000000002</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A195" s="6">
+      <c r="A195" s="5">
         <v>0.96499999999999997</v>
       </c>
-      <c r="B195" s="6">
+      <c r="B195" s="5">
         <v>4.1231499999999999</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A196" s="6">
+      <c r="A196" s="5">
         <v>0.97</v>
       </c>
-      <c r="B196" s="6">
+      <c r="B196" s="5">
         <v>4.1285999999999996</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A197" s="6">
+      <c r="A197" s="5">
         <v>0.97499999999999998</v>
       </c>
-      <c r="B197" s="6">
+      <c r="B197" s="5">
         <v>4.1349213000000002</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A198" s="6">
+      <c r="A198" s="5">
         <v>0.98</v>
       </c>
-      <c r="B198" s="6">
+      <c r="B198" s="5">
         <v>4.1422999999999996</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A199" s="6">
+      <c r="A199" s="5">
         <v>0.98499999999999999</v>
       </c>
-      <c r="B199" s="6">
+      <c r="B199" s="5">
         <v>4.1509608</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A200" s="6">
+      <c r="A200" s="5">
         <v>0.99</v>
       </c>
-      <c r="B200" s="6">
+      <c r="B200" s="5">
         <v>4.1612</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A201" s="6">
+      <c r="A201" s="5">
         <v>0.995</v>
       </c>
-      <c r="B201" s="6">
+      <c r="B201" s="5">
         <v>4.1732202999999997</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A202" s="6">
+      <c r="A202" s="5">
         <v>1</v>
       </c>
-      <c r="B202" s="6">
+      <c r="B202" s="5">
         <v>4.1895499999999997</v>
       </c>
     </row>
@@ -2276,88 +2218,1703 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:B202"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2.174459866666667E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="B3">
+        <v>2.16624999E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>0.01</v>
+      </c>
+      <c r="B4">
+        <v>2.158040113333334E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="B5">
+        <v>2.149830236666667E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>0.02</v>
+      </c>
+      <c r="B6">
+        <v>2.1416203599999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="B7">
+        <v>2.1334104833333339E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>0.03</v>
+      </c>
+      <c r="B8">
+        <v>2.1252006066666669E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="B9">
+        <v>2.1169907299999999E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>0.04</v>
+      </c>
+      <c r="B10">
+        <v>2.1087808533333339E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="B11">
+        <v>2.1005709766666669E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>0.05</v>
+      </c>
+      <c r="B12">
+        <v>2.0923611000000002E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>5.5E-2</v>
+      </c>
+      <c r="B13">
+        <v>2.0841512233333331E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>0.06</v>
+      </c>
+      <c r="B14">
+        <v>2.0759413466666671E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="B15">
+        <v>2.0677314700000001E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="B16">
+        <v>2.0595215933333331E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="B17">
+        <v>2.0513117166666671E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>0.08</v>
+      </c>
+      <c r="B18">
+        <v>2.0431018400000001E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="B19">
+        <v>2.034891963333333E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>0.09</v>
+      </c>
+      <c r="B20">
+        <v>2.026682086666667E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>9.5000000000000001E-2</v>
+      </c>
+      <c r="B21">
+        <v>2.01847221E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>0.1</v>
+      </c>
+      <c r="B22">
+        <v>2.010262333333333E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>0.105</v>
+      </c>
+      <c r="B23">
+        <v>2.002052456666667E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>0.11</v>
+      </c>
+      <c r="B24">
+        <v>1.9938425799999999E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>0.115</v>
+      </c>
+      <c r="B25">
+        <v>1.9856327033333329E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>0.12</v>
+      </c>
+      <c r="B26">
+        <v>1.9774228266666669E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>0.125</v>
+      </c>
+      <c r="B27">
+        <v>1.9692129499999999E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>0.13</v>
+      </c>
+      <c r="B28">
+        <v>1.9610030733333339E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>0.13500000000000001</v>
+      </c>
+      <c r="B29">
+        <v>1.9527931966666669E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="B30">
+        <v>1.9445833199999998E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="B31">
+        <v>1.9363734433333332E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>0.15</v>
+      </c>
+      <c r="B32">
+        <v>1.9281635666666672E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>0.155</v>
+      </c>
+      <c r="B33">
+        <v>1.9199536900000001E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>0.16</v>
+      </c>
+      <c r="B34">
+        <v>1.9117438133333331E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="B35">
+        <v>1.9035339366666671E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>0.17</v>
+      </c>
+      <c r="B36">
+        <v>1.8953240600000001E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="B37">
+        <v>1.887114183333333E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>0.18</v>
+      </c>
+      <c r="B38">
+        <v>1.8789043066666671E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>0.185</v>
+      </c>
+      <c r="B39">
+        <v>1.87069443E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>0.19</v>
+      </c>
+      <c r="B40">
+        <v>1.862484553333333E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>0.19500000000000001</v>
+      </c>
+      <c r="B41">
+        <v>1.854274676666667E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>0.2</v>
+      </c>
+      <c r="B42">
+        <v>1.8460648E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="B43">
+        <v>1.8437444733333329E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>0.21</v>
+      </c>
+      <c r="B44">
+        <v>1.8414241466666662E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>0.215</v>
+      </c>
+      <c r="B45">
+        <v>1.8391038200000001E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>0.22</v>
+      </c>
+      <c r="B46">
+        <v>1.836783493333333E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="B47">
+        <v>1.834463166666667E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>0.23</v>
+      </c>
+      <c r="B48">
+        <v>1.8321428399999999E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>0.23499999999999999</v>
+      </c>
+      <c r="B49">
+        <v>1.8298225133333328E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>0.24</v>
+      </c>
+      <c r="B50">
+        <v>1.8275021866666671E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>0.245</v>
+      </c>
+      <c r="B51">
+        <v>1.8251818600000001E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>0.25</v>
+      </c>
+      <c r="B52">
+        <v>1.822861533333333E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>0.255</v>
+      </c>
+      <c r="B53">
+        <v>1.8205412066666669E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>0.26</v>
+      </c>
+      <c r="B54">
+        <v>1.8182208799999999E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>0.26500000000000001</v>
+      </c>
+      <c r="B55">
+        <v>1.8159005533333331E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>0.27</v>
+      </c>
+      <c r="B56">
+        <v>1.8135802266666671E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="B57">
+        <v>1.8112599E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="B58">
+        <v>1.8089395733333329E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="B59">
+        <v>1.8066192466666669E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="B60">
+        <v>1.8042989200000002E-2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>0.29499999999999998</v>
+      </c>
+      <c r="B61">
+        <v>1.8019785933333331E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>0.3</v>
+      </c>
+      <c r="B62">
+        <v>1.799658266666667E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>0.30499999999999999</v>
+      </c>
+      <c r="B63">
+        <v>1.79733794E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>0.31</v>
+      </c>
+      <c r="B64">
+        <v>1.7950176133333329E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>0.315</v>
+      </c>
+      <c r="B65">
+        <v>1.7926972866666668E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>0.32</v>
+      </c>
+      <c r="B66">
+        <v>1.7903769600000001E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="B67">
+        <v>1.788056633333333E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>0.33</v>
+      </c>
+      <c r="B68">
+        <v>1.785736306666667E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>0.33500000000000002</v>
+      </c>
+      <c r="B69">
+        <v>1.7834159799999999E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>0.34</v>
+      </c>
+      <c r="B70">
+        <v>1.7810956533333339E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>0.34499999999999997</v>
+      </c>
+      <c r="B71">
+        <v>1.7787753266666671E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>0.35</v>
+      </c>
+      <c r="B72">
+        <v>1.776455E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>0.35499999999999998</v>
+      </c>
+      <c r="B73">
+        <v>1.7758608666666668E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>0.36</v>
+      </c>
+      <c r="B74">
+        <v>1.7752667333333329E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>0.36499999999999999</v>
+      </c>
+      <c r="B75">
+        <v>1.7746726000000001E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>0.37</v>
+      </c>
+      <c r="B76">
+        <v>1.7740784666666669E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>0.375</v>
+      </c>
+      <c r="B77">
+        <v>1.773484333333333E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>0.38</v>
+      </c>
+      <c r="B78">
+        <v>1.7728902000000001E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>0.38500000000000001</v>
+      </c>
+      <c r="B79">
+        <v>1.7722960666666669E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>0.39</v>
+      </c>
+      <c r="B80">
+        <v>1.771701933333333E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="B81">
+        <v>1.7711078000000002E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>0.4</v>
+      </c>
+      <c r="B82">
+        <v>1.770513666666667E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>0.40500000000000003</v>
+      </c>
+      <c r="B83">
+        <v>1.7699195333333331E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>0.41</v>
+      </c>
+      <c r="B84">
+        <v>1.7693253999999999E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>0.41499999999999998</v>
+      </c>
+      <c r="B85">
+        <v>1.768731266666667E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>0.42</v>
+      </c>
+      <c r="B86">
+        <v>1.7681371333333331E-2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>0.42499999999999999</v>
+      </c>
+      <c r="B87">
+        <v>1.7675429999999999E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>0.43</v>
+      </c>
+      <c r="B88">
+        <v>1.766948866666667E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>0.435</v>
+      </c>
+      <c r="B89">
+        <v>1.7663547333333331E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>0.44</v>
+      </c>
+      <c r="B90">
+        <v>1.7657605999999999E-2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>0.44500000000000001</v>
+      </c>
+      <c r="B91">
+        <v>1.7651664666666671E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>0.45</v>
+      </c>
+      <c r="B92">
+        <v>1.7645723333333339E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="B93">
+        <v>1.7639782E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>0.46</v>
+      </c>
+      <c r="B94">
+        <v>1.7633840666666671E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="B95">
+        <v>1.7627899333333339E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>0.47</v>
+      </c>
+      <c r="B96">
+        <v>1.7621958E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="B97">
+        <v>1.7616016666666671E-2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>0.48</v>
+      </c>
+      <c r="B98">
+        <v>1.7610075333333329E-2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>0.48499999999999999</v>
+      </c>
+      <c r="B99">
+        <v>1.7604134E-2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>0.49</v>
+      </c>
+      <c r="B100">
+        <v>1.7598192666666668E-2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <v>0.495</v>
+      </c>
+      <c r="B101">
+        <v>1.7592251333333329E-2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <v>0.5</v>
+      </c>
+      <c r="B102">
+        <v>1.7586310000000001E-2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>0.505</v>
+      </c>
+      <c r="B103">
+        <v>1.75858801E-2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <v>0.51</v>
+      </c>
+      <c r="B104">
+        <v>1.7585450200000002E-2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="B105">
+        <v>1.75850203E-2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <v>0.52</v>
+      </c>
+      <c r="B106">
+        <v>1.7584590399999999E-2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A107">
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="B107">
+        <v>1.7584160500000001E-2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A108">
+        <v>0.53</v>
+      </c>
+      <c r="B108">
+        <v>1.75837306E-2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A109">
+        <v>0.53500000000000003</v>
+      </c>
+      <c r="B109">
+        <v>1.7583300699999999E-2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A110">
+        <v>0.54</v>
+      </c>
+      <c r="B110">
+        <v>1.7582870800000001E-2</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111">
+        <v>0.54500000000000004</v>
+      </c>
+      <c r="B111">
+        <v>1.7582440899999999E-2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="B112">
+        <v>1.7582011000000002E-2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <v>0.55500000000000005</v>
+      </c>
+      <c r="B113">
+        <v>1.75815811E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="B114">
+        <v>1.7581151199999999E-2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <v>0.56499999999999995</v>
+      </c>
+      <c r="B115">
+        <v>1.7580721300000001E-2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="B116">
+        <v>1.75802914E-2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <v>0.57499999999999996</v>
+      </c>
+      <c r="B117">
+        <v>1.7579861499999998E-2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="B118">
+        <v>1.7579431600000001E-2</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <v>0.58499999999999996</v>
+      </c>
+      <c r="B119">
+        <v>1.7579001699999999E-2</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A120">
+        <v>0.59</v>
+      </c>
+      <c r="B120">
+        <v>1.7578571800000001E-2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <v>0.59499999999999997</v>
+      </c>
+      <c r="B121">
+        <v>1.75781419E-2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <v>0.6</v>
+      </c>
+      <c r="B122">
+        <v>1.7577711999999999E-2</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A123">
+        <v>0.60499999999999998</v>
+      </c>
+      <c r="B123">
+        <v>1.7577282100000001E-2</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A124">
+        <v>0.61</v>
+      </c>
+      <c r="B124">
+        <v>1.75768522E-2</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A125">
+        <v>0.61499999999999999</v>
+      </c>
+      <c r="B125">
+        <v>1.7576422299999998E-2</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A126">
+        <v>0.62</v>
+      </c>
+      <c r="B126">
+        <v>1.75759924E-2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A127">
+        <v>0.625</v>
+      </c>
+      <c r="B127">
+        <v>1.7575562499999999E-2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <v>0.63</v>
+      </c>
+      <c r="B128">
+        <v>1.7575132600000001E-2</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="B129">
+        <v>1.75747027E-2</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <v>0.64</v>
+      </c>
+      <c r="B130">
+        <v>1.7574272799999999E-2</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <v>0.64500000000000002</v>
+      </c>
+      <c r="B131">
+        <v>1.7573842900000001E-2</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <v>0.65</v>
+      </c>
+      <c r="B132">
+        <v>1.7573413E-2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A133">
+        <v>0.65500000000000003</v>
+      </c>
+      <c r="B133">
+        <v>1.7582639166666671E-2</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A134">
+        <v>0.66</v>
+      </c>
+      <c r="B134">
+        <v>1.7591865333333331E-2</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A135">
+        <v>0.66500000000000004</v>
+      </c>
+      <c r="B135">
+        <v>1.7601091499999999E-2</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A136">
+        <v>0.67</v>
+      </c>
+      <c r="B136">
+        <v>1.761031766666667E-2</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A137">
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="B137">
+        <v>1.7619543833333331E-2</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A138">
+        <v>0.68</v>
+      </c>
+      <c r="B138">
+        <v>1.7628769999999998E-2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A139">
+        <v>0.68500000000000005</v>
+      </c>
+      <c r="B139">
+        <v>1.763799616666667E-2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A140">
+        <v>0.69</v>
+      </c>
+      <c r="B140">
+        <v>1.764722233333333E-2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A141">
+        <v>0.69499999999999995</v>
+      </c>
+      <c r="B141">
+        <v>1.7656448500000001E-2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A142">
+        <v>0.7</v>
+      </c>
+      <c r="B142">
+        <v>1.7665674666666669E-2</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A143">
+        <v>0.70499999999999996</v>
+      </c>
+      <c r="B143">
+        <v>1.767490083333333E-2</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A144">
+        <v>0.71</v>
+      </c>
+      <c r="B144">
+        <v>1.7684127000000001E-2</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A145">
+        <v>0.71499999999999997</v>
+      </c>
+      <c r="B145">
+        <v>1.7693353166666669E-2</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A146">
+        <v>0.72</v>
+      </c>
+      <c r="B146">
+        <v>1.7702579333333329E-2</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A147">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="B147">
+        <v>1.77118055E-2</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A148">
+        <v>0.73</v>
+      </c>
+      <c r="B148">
+        <v>1.7721031666666671E-2</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A149">
+        <v>0.73499999999999999</v>
+      </c>
+      <c r="B149">
+        <v>1.7730257833333329E-2</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A150">
+        <v>0.74</v>
+      </c>
+      <c r="B150">
+        <v>1.7739484E-2</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A151">
+        <v>0.745</v>
+      </c>
+      <c r="B151">
+        <v>1.7748710166666671E-2</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A152">
+        <v>0.75</v>
+      </c>
+      <c r="B152">
+        <v>1.7757936333333339E-2</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A153">
+        <v>0.755</v>
+      </c>
+      <c r="B153">
+        <v>1.7767162499999999E-2</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A154">
+        <v>0.76</v>
+      </c>
+      <c r="B154">
+        <v>1.777638866666667E-2</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A155">
+        <v>0.76500000000000001</v>
+      </c>
+      <c r="B155">
+        <v>1.7785614833333331E-2</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A156">
+        <v>0.77</v>
+      </c>
+      <c r="B156">
+        <v>1.7794840999999999E-2</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A157">
+        <v>0.77500000000000002</v>
+      </c>
+      <c r="B157">
+        <v>1.780406716666667E-2</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A158">
+        <v>0.78</v>
+      </c>
+      <c r="B158">
+        <v>1.7813293333333331E-2</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A159">
+        <v>0.78500000000000003</v>
+      </c>
+      <c r="B159">
+        <v>1.7822519500000002E-2</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A160">
+        <v>0.79</v>
+      </c>
+      <c r="B160">
+        <v>1.7831745666666669E-2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A161">
+        <v>0.79500000000000004</v>
+      </c>
+      <c r="B161">
+        <v>1.784097183333333E-2</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A162">
+        <v>0.8</v>
+      </c>
+      <c r="B162">
+        <v>1.7850198000000001E-2</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A163">
+        <v>0.80500000000000005</v>
+      </c>
+      <c r="B163">
+        <v>1.7871494299999999E-2</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A164">
+        <v>0.81</v>
+      </c>
+      <c r="B164">
+        <v>1.78927906E-2</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A165">
+        <v>0.81499999999999995</v>
+      </c>
+      <c r="B165">
+        <v>1.7914086900000001E-2</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A166">
+        <v>0.82</v>
+      </c>
+      <c r="B166">
+        <v>1.7935383199999998E-2</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A167">
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="B167">
+        <v>1.7956679499999999E-2</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A168">
+        <v>0.83</v>
+      </c>
+      <c r="B168">
+        <v>1.79779758E-2</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A169">
+        <v>0.83499999999999996</v>
+      </c>
+      <c r="B169">
+        <v>1.7999272100000002E-2</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A170">
+        <v>0.84</v>
+      </c>
+      <c r="B170">
+        <v>1.8020568399999999E-2</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A171">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="B171">
+        <v>1.80418647E-2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A172">
+        <v>0.85</v>
+      </c>
+      <c r="B172">
+        <v>1.8063161000000001E-2</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A173">
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="B173">
+        <v>1.8084457299999999E-2</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A174">
+        <v>0.86</v>
+      </c>
+      <c r="B174">
+        <v>1.81057536E-2</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A175">
+        <v>0.86499999999999999</v>
+      </c>
+      <c r="B175">
+        <v>1.8127049900000001E-2</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A176">
+        <v>0.87</v>
+      </c>
+      <c r="B176">
+        <v>1.8148346199999998E-2</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A177">
+        <v>0.875</v>
+      </c>
+      <c r="B177">
+        <v>1.8169642499999999E-2</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A178">
+        <v>0.88</v>
+      </c>
+      <c r="B178">
+        <v>1.8190938800000001E-2</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A179">
+        <v>0.88500000000000001</v>
+      </c>
+      <c r="B179">
+        <v>1.8212235100000002E-2</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A180">
+        <v>0.89</v>
+      </c>
+      <c r="B180">
+        <v>1.8233531399999999E-2</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A181">
+        <v>0.89500000000000002</v>
+      </c>
+      <c r="B181">
+        <v>1.82548277E-2</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A182">
+        <v>0.9</v>
+      </c>
+      <c r="B182">
+        <v>1.8276124000000001E-2</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A183">
+        <v>0.90500000000000003</v>
+      </c>
+      <c r="B183">
+        <v>1.8297420299999999E-2</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A184">
+        <v>0.91</v>
+      </c>
+      <c r="B184">
+        <v>1.83187166E-2</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A185">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="B185">
+        <v>1.8340012900000001E-2</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A186">
+        <v>0.92</v>
+      </c>
+      <c r="B186">
+        <v>1.8361309199999998E-2</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A187">
+        <v>0.92500000000000004</v>
+      </c>
+      <c r="B187">
+        <v>1.83826055E-2</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A188">
+        <v>0.93</v>
+      </c>
+      <c r="B188">
+        <v>1.8403901800000001E-2</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A189">
+        <v>0.93500000000000005</v>
+      </c>
+      <c r="B189">
+        <v>1.8425198100000002E-2</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A190">
+        <v>0.94</v>
+      </c>
+      <c r="B190">
+        <v>1.8446494399999999E-2</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A191">
+        <v>0.94499999999999995</v>
+      </c>
+      <c r="B191">
+        <v>1.84677907E-2</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A192">
+        <v>0.95</v>
+      </c>
+      <c r="B192">
+        <v>1.8489087000000001E-2</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A193">
+        <v>0.95499999999999996</v>
+      </c>
+      <c r="B193">
+        <v>1.8510383299999999E-2</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A194">
+        <v>0.96</v>
+      </c>
+      <c r="B194">
+        <v>1.85316796E-2</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A195">
+        <v>0.96499999999999997</v>
+      </c>
+      <c r="B195">
+        <v>1.8552975900000001E-2</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A196">
+        <v>0.97</v>
+      </c>
+      <c r="B196">
+        <v>1.8574272199999999E-2</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A197">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="B197">
+        <v>1.85955685E-2</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A198">
+        <v>0.98</v>
+      </c>
+      <c r="B198">
+        <v>1.8616864800000001E-2</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A199">
+        <v>0.98499999999999999</v>
+      </c>
+      <c r="B199">
+        <v>1.8638161100000002E-2</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A200">
+        <v>0.99</v>
+      </c>
+      <c r="B200">
+        <v>1.8659457399999999E-2</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A201">
+        <v>0.995</v>
+      </c>
+      <c r="B201">
+        <v>1.86807537E-2</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A202">
+        <v>1</v>
+      </c>
+      <c r="B202">
+        <v>1.8702050000000001E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="3"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="5">
         <v>0.05</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="5">
         <v>2.0923611000000002E-2</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="6">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5">
         <v>0.2</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="5">
         <v>1.8460648E-2</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="6">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="5">
         <v>0.35</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>1.776455E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="6">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="5">
         <v>0.5</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <v>1.7586310000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="5">
         <v>0.65</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <v>1.7573413E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="6">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="5">
         <v>0.8</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <v>1.7850198000000001E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="6">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="5">
         <v>0.95</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <v>1.8489087000000001E-2</v>
       </c>
     </row>

</xml_diff>